<commit_message>
Rose plot - Draft2
</commit_message>
<xml_diff>
--- a/public_security/visualizations/rose_diagram/input/toques_queda.xlsx
+++ b/public_security/visualizations/rose_diagram/input/toques_queda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luismunoz/Documents/Documents MacBook Air/git/Police-Violence/public_security/visualizations/rose_diagram/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F8CB6C-D04B-564E-A0E6-7FBD59DA103B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{181B1DB4-0454-B947-BF29-04832C9F5695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4309,7 +4309,7 @@
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.1640625" customWidth="1"/>
     <col min="3" max="3" width="30.33203125" customWidth="1"/>
-    <col min="4" max="4" width="32.33203125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" customWidth="1"/>
     <col min="5" max="7" width="17.33203125" customWidth="1"/>
     <col min="8" max="8" width="14.1640625" customWidth="1"/>
     <col min="9" max="10" width="16.33203125" customWidth="1"/>

</xml_diff>